<commit_message>
Update Zero Trust page content and revert port to 3002
</commit_message>
<xml_diff>
--- a/noti/별표7_망분리 대체 정보보호통제.xlsx
+++ b/noti/별표7_망분리 대체 정보보호통제.xlsx
@@ -5,17 +5,30 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunhyeok/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunhyeok/portfolio/noti/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF2067F-55BA-9940-B77F-B31E047822A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A61885C-4BC4-9249-8623-F1568A3381BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37360" yWindow="-2640" windowWidth="14400" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37360" yWindow="-620" windowWidth="22060" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시트1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -672,27 +685,27 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -915,8 +928,9 @@
   <dimension ref="B1:G1005"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="6" max="6" width="35" customWidth="1"/>
-    <col min="7" max="7" width="53.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="6" max="6" width="46.5" customWidth="1"/>
+    <col min="7" max="7" width="57.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -952,55 +966,55 @@
       <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="18"/>
-      <c r="F4" s="19"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="18"/>
       <c r="G4" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="23" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="5">
         <v>1</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="19"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="18"/>
       <c r="G5" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="16"/>
+      <c r="B6" s="15"/>
       <c r="C6" s="5">
         <v>2</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="19"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="18"/>
       <c r="G6" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B7" s="15"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="5">
         <v>3</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="19"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="6" t="s">
         <v>11</v>
       </c>
@@ -1012,25 +1026,25 @@
       <c r="C8" s="8">
         <v>4</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="18"/>
-      <c r="F8" s="19"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="9" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B9" s="15"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="8">
         <v>5</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="18"/>
-      <c r="F9" s="19"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="18"/>
       <c r="G9" s="10" t="s">
         <v>16</v>
       </c>
@@ -1042,39 +1056,39 @@
       <c r="C10" s="8">
         <v>6</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="18"/>
-      <c r="F10" s="19"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="10" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B11" s="16"/>
+      <c r="B11" s="15"/>
       <c r="C11" s="8">
         <v>7</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="10" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B12" s="15"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="8">
         <v>8</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="18"/>
       <c r="G12" s="10" t="s">
         <v>23</v>
       </c>
@@ -1086,67 +1100,67 @@
       <c r="C13" s="8">
         <v>9</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="18"/>
-      <c r="F13" s="19"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="18"/>
       <c r="G13" s="11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B14" s="16"/>
+      <c r="B14" s="15"/>
       <c r="C14" s="8">
         <v>10</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="F14" s="19"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="18"/>
       <c r="G14" s="11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="16"/>
+      <c r="B15" s="15"/>
       <c r="C15" s="8">
         <v>11</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="18"/>
       <c r="G15" s="11" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B16" s="16"/>
+      <c r="B16" s="15"/>
       <c r="C16" s="8">
         <v>12</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="18"/>
-      <c r="F16" s="19"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="18"/>
       <c r="G16" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B17" s="15"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="8">
         <v>13</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="18"/>
-      <c r="F17" s="19"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="18"/>
       <c r="G17" s="11" t="s">
         <v>34</v>
       </c>
@@ -1161,7 +1175,7 @@
       <c r="D18" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="21" t="s">
         <v>5</v>
       </c>
       <c r="F18" s="11" t="s">
@@ -1172,12 +1186,12 @@
       </c>
     </row>
     <row r="19" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B19" s="16"/>
+      <c r="B19" s="15"/>
       <c r="C19" s="8">
         <v>15</v>
       </c>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
       <c r="F19" s="11" t="s">
         <v>39</v>
       </c>
@@ -1186,12 +1200,12 @@
       </c>
     </row>
     <row r="20" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B20" s="16"/>
+      <c r="B20" s="15"/>
       <c r="C20" s="8">
         <v>16</v>
       </c>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
       <c r="F20" s="11" t="s">
         <v>41</v>
       </c>
@@ -1200,12 +1214,12 @@
       </c>
     </row>
     <row r="21" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B21" s="16"/>
+      <c r="B21" s="15"/>
       <c r="C21" s="8">
         <v>17</v>
       </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="16"/>
       <c r="F21" s="11" t="s">
         <v>43</v>
       </c>
@@ -1214,11 +1228,11 @@
       </c>
     </row>
     <row r="22" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B22" s="16"/>
+      <c r="B22" s="15"/>
       <c r="C22" s="8">
         <v>18</v>
       </c>
-      <c r="D22" s="16"/>
+      <c r="D22" s="15"/>
       <c r="E22" s="8" t="s">
         <v>45</v>
       </c>
@@ -1230,12 +1244,12 @@
       </c>
     </row>
     <row r="23" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B23" s="16"/>
+      <c r="B23" s="15"/>
       <c r="C23" s="8">
         <v>14</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="24" t="s">
+      <c r="D23" s="15"/>
+      <c r="E23" s="21" t="s">
         <v>48</v>
       </c>
       <c r="F23" s="11" t="s">
@@ -1246,12 +1260,12 @@
       </c>
     </row>
     <row r="24" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B24" s="16"/>
+      <c r="B24" s="15"/>
       <c r="C24" s="8">
         <v>15</v>
       </c>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="11" t="s">
         <v>50</v>
       </c>
@@ -1260,12 +1274,12 @@
       </c>
     </row>
     <row r="25" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B25" s="16"/>
+      <c r="B25" s="15"/>
       <c r="C25" s="8">
         <v>16</v>
       </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
       <c r="F25" s="11" t="s">
         <v>51</v>
       </c>
@@ -1274,12 +1288,12 @@
       </c>
     </row>
     <row r="26" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B26" s="16"/>
+      <c r="B26" s="15"/>
       <c r="C26" s="8">
         <v>17</v>
       </c>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
       <c r="F26" s="11" t="s">
         <v>53</v>
       </c>
@@ -1288,12 +1302,12 @@
       </c>
     </row>
     <row r="27" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B27" s="16"/>
+      <c r="B27" s="15"/>
       <c r="C27" s="8">
         <v>18</v>
       </c>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
       <c r="F27" s="11" t="s">
         <v>55</v>
       </c>
@@ -1302,135 +1316,135 @@
       </c>
     </row>
     <row r="28" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B28" s="16"/>
+      <c r="B28" s="15"/>
       <c r="C28" s="8">
         <v>19</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="F28" s="19"/>
+      <c r="F28" s="18"/>
       <c r="G28" s="11" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B29" s="16"/>
+      <c r="B29" s="15"/>
       <c r="C29" s="8">
         <v>20</v>
       </c>
-      <c r="D29" s="15"/>
-      <c r="E29" s="22" t="s">
+      <c r="D29" s="16"/>
+      <c r="E29" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="F29" s="19"/>
+      <c r="F29" s="18"/>
       <c r="G29" s="13" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B30" s="16"/>
+      <c r="B30" s="15"/>
       <c r="C30" s="8">
         <v>21</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="F30" s="19"/>
+      <c r="F30" s="18"/>
       <c r="G30" s="13" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B31" s="16"/>
+      <c r="B31" s="15"/>
       <c r="C31" s="8">
         <v>22</v>
       </c>
-      <c r="D31" s="15"/>
-      <c r="E31" s="22" t="s">
+      <c r="D31" s="16"/>
+      <c r="E31" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="F31" s="19"/>
+      <c r="F31" s="18"/>
       <c r="G31" s="13" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B32" s="16"/>
+      <c r="B32" s="15"/>
       <c r="C32" s="8">
         <v>23</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="E32" s="22" t="s">
+      <c r="E32" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="F32" s="19"/>
+      <c r="F32" s="18"/>
       <c r="G32" s="13" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B33" s="16"/>
+      <c r="B33" s="15"/>
       <c r="C33" s="8">
         <v>24</v>
       </c>
-      <c r="D33" s="16"/>
-      <c r="E33" s="22" t="s">
+      <c r="D33" s="15"/>
+      <c r="E33" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="F33" s="19"/>
+      <c r="F33" s="18"/>
       <c r="G33" s="13" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B34" s="16"/>
+      <c r="B34" s="15"/>
       <c r="C34" s="8">
         <v>25</v>
       </c>
-      <c r="D34" s="15"/>
-      <c r="E34" s="22" t="s">
+      <c r="D34" s="16"/>
+      <c r="E34" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="F34" s="19"/>
+      <c r="F34" s="18"/>
       <c r="G34" s="13" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="35" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B35" s="16"/>
+      <c r="B35" s="15"/>
       <c r="C35" s="8">
         <v>26</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E35" s="22" t="s">
+      <c r="E35" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="F35" s="19"/>
+      <c r="F35" s="18"/>
       <c r="G35" s="10" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="36" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B36" s="15"/>
+      <c r="B36" s="16"/>
       <c r="C36" s="8">
         <v>27</v>
       </c>
-      <c r="D36" s="15"/>
-      <c r="E36" s="22" t="s">
+      <c r="D36" s="16"/>
+      <c r="E36" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F36" s="19"/>
+      <c r="F36" s="18"/>
       <c r="G36" s="10" t="s">
         <v>76</v>
       </c>
@@ -9189,25 +9203,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D18:D27"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="E23:E27"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="E31:F31"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B13:B17"/>
@@ -9224,6 +9219,25 @@
     <mergeCell ref="D12:F12"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:D27"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="E23:E27"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E36:F36"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>